<commit_message>
fix(productos): Fase A — impresión A4 COMPLETA en 147 hojas de 11 kits de tareas que el generador había dejado en A4 mínimo (sin ajuste al ancho, pie ni cabecera repetida); el post-proceso y el censo exigen ahora A4 + ajuste + pie en hojas de datos (paperSize 9 basta en Instrucciones)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-bar/08-apertura-cierre-negocio.xlsx
+++ b/astro-site/public/dl/kit-tareas-bar/08-apertura-cierre-negocio.xlsx
@@ -13,7 +13,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$A$20</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Apertura del Negocio'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Apertura del Negocio'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Cierre del Negocio'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Cierre del Negocio'!$A$1:$H$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -710,7 +712,7 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
@@ -1199,8 +1201,16 @@
       <formula1>"✓,✗,—"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1209,7 +1219,7 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
@@ -1638,7 +1648,15 @@
       <formula1>"✓,✗,—"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>